<commit_message>
Expand selection competition analysis across category keywords and stores
</commit_message>
<xml_diff>
--- a/skills/amazon-product-direction/assets/亚马逊选品表.xlsx
+++ b/skills/amazon-product-direction/assets/亚马逊选品表.xlsx
@@ -2,12 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="类目判断" sheetId="1" r:id="R6800b8ffd92844ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="选品表" sheetId="2" r:id="R2ce54395bfe4494e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="市场与关键词" sheetId="3" r:id="R5d79c646d08d416b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="差评分析" sheetId="4" r:id="Rf407c79a65dc4a28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="初筛规则" sheetId="5" r:id="R3ee55af5e56e4973"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="选品方法" sheetId="6" r:id="R5db19699271e4faf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="类目判断" sheetId="1" r:id="R7d6832fb5eb946d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="选品表" sheetId="2" r:id="R1b4b9ba6797e4731"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="市场与关键词" sheetId="3" r:id="Ra9164af1baa4444b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="差评分析" sheetId="4" r:id="R349e7d6278ac4e01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="初筛规则" sheetId="5" r:id="Rad5651cfa88144ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="选品方法" sheetId="6" r:id="Rb4cdac618bae4632"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="竞争分析" sheetId="7" r:id="Rfb5ae4cf27644542"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,13 +19,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="6">
+  <x:numFmts count="7">
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="201" formatCode="0.0"/>
     <x:numFmt numFmtId="202" formatCode="#,##0.00"/>
     <x:numFmt numFmtId="203" formatCode="0.0%"/>
     <x:numFmt numFmtId="204" formatCode="0%"/>
     <x:numFmt numFmtId="205" formatCode="0"/>
+    <x:numFmt numFmtId="206" formatCode="0.00"/>
   </x:numFmts>
   <x:fonts count="5">
     <x:font>
@@ -114,7 +116,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="48">
+  <x:cellXfs count="51">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -250,6 +252,15 @@
     </x:xf>
     <x:xf numFmtId="204" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -416,6 +427,30 @@
     <x:tableColumn id="17" name="评分依据"/>
     <x:tableColumn id="18" name="工具来源"/>
     <x:tableColumn id="19" name="核查日期"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CompetitionEvidence" displayName="CompetitionEvidence" ref="A5:O24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:O24"/>
+  <x:tableColumns count="15">
+    <x:tableColumn id="1" name="分析层级"/>
+    <x:tableColumn id="2" name="选品分析方法"/>
+    <x:tableColumn id="3" name="研究对象"/>
+    <x:tableColumn id="4" name="指标"/>
+    <x:tableColumn id="5" name="观察／数值"/>
+    <x:tableColumn id="6" name="单位"/>
+    <x:tableColumn id="7" name="样本范围"/>
+    <x:tableColumn id="8" name="统计定义"/>
+    <x:tableColumn id="9" name="数据覆盖"/>
+    <x:tableColumn id="10" name="判断规则"/>
+    <x:tableColumn id="11" name="信号／分析"/>
+    <x:tableColumn id="12" name="数据来源"/>
+    <x:tableColumn id="13" name="采集日期"/>
+    <x:tableColumn id="14" name="数据状态"/>
+    <x:tableColumn id="15" name="限制与缺口"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -1216,7 +1251,7 @@
         <x:v>最终进入结论</x:v>
       </x:c>
       <x:c r="B48" s="21" t="str">
-        <x:f>IF(LEFT(B45,2)="否决","淘汰（利润否决）",IF(OR(B47="淘汰",B47="暂缓"),B47,IF($B$19="初筛","仅初筛，待深度验证",IF(B45&lt;&gt;"达标","待验证",IF(NOT(ISNUMBER(B50)),"待验证",IF(B50&lt;'初筛规则'!$B$14,"暂缓（初筛）",IF(B46="已确认相关风险","暂缓（专利风险）",IF(OR(B21&lt;&gt;$B$12,B23&lt;&gt;$B$12,B33&lt;&gt;$B$12,B29&lt;&gt;$B$12,B32="",B39="",B40="",B41="",B42="",B53="待补初筛数据",B52="待补方法与依据",B46="待核查",B46="发现相关专利"),"待验证",B47))))))))</x:f>
+        <x:f>IF(LEFT(B45,2)="否决","淘汰（利润否决）",IF(OR(B47="淘汰",B47="暂缓"),B47,IF($B$19="初筛","仅初筛，待深度验证",IF(B45&lt;&gt;"达标","待验证",IF(NOT(ISNUMBER(B50)),"待验证",IF(B50&lt;'初筛规则'!$B$14,"暂缓（初筛）",IF(B46="已确认相关风险","暂缓（专利风险）",IF(OR(B21&lt;&gt;$B$12,B23&lt;&gt;$B$12,B33&lt;&gt;$B$12,B29&lt;&gt;$B$12,B32="",B55="",B56="",B57="",B39="",B40="",B41="",B42="",B53="待补初筛数据",B52="待补方法与依据",B46="待核查",B46="发现相关专利"),"待验证",B47))))))))</x:f>
         <x:v>仅初筛，待深度验证</x:v>
       </x:c>
       <x:c r="C48" s="21" t="str">
@@ -1311,6 +1346,66 @@
       </x:c>
       <x:c r="D54" s="45" t="str">
         <x:v>追溯选品方法与评分依据</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="60" customHeight="1">
+      <x:c r="A55" s="45" t="str">
+        <x:v>类目竞争结论</x:v>
+      </x:c>
+      <x:c r="B55" s="45"/>
+      <x:c r="C55" s="45" t="str">
+        <x:v>Top100与Top50分别记录，至少一条可得路线</x:v>
+      </x:c>
+      <x:c r="D55" s="45" t="str">
+        <x:v>见竞争分析页与逐项来源</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="60" customHeight="1">
+      <x:c r="A56" s="45" t="str">
+        <x:v>关键词竞价结论</x:v>
+      </x:c>
+      <x:c r="B56" s="45"/>
+      <x:c r="C56" s="45" t="str">
+        <x:v>后台建议竞价、实际CPC与利润承受力</x:v>
+      </x:c>
+      <x:c r="D56" s="45" t="str">
+        <x:v>见竞争分析页与逐项来源</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="60" customHeight="1">
+      <x:c r="A57" s="45" t="str">
+        <x:v>竞品店铺实力</x:v>
+      </x:c>
+      <x:c r="B57" s="45"/>
+      <x:c r="C57" s="45" t="str">
+        <x:v>商品评价、商标、地区、SKU、内容、站外</x:v>
+      </x:c>
+      <x:c r="D57" s="45" t="str">
+        <x:v>见竞争分析页与逐项来源</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="60" customHeight="1">
+      <x:c r="A58" s="45" t="str">
+        <x:v>竞争工具路径</x:v>
+      </x:c>
+      <x:c r="B58" s="45"/>
+      <x:c r="C58" s="45" t="str">
+        <x:v>Sorftime或Flapen＋ASINSIGHT及覆盖</x:v>
+      </x:c>
+      <x:c r="D58" s="45" t="str">
+        <x:v>见竞争分析页与逐项来源</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="60" customHeight="1">
+      <x:c r="A59" s="45" t="str">
+        <x:v>竞争证据缺口</x:v>
+      </x:c>
+      <x:c r="B59" s="45"/>
+      <x:c r="C59" s="45" t="str">
+        <x:v>注明缺字段、样本、权限或统计定义</x:v>
+      </x:c>
+      <x:c r="D59" s="45" t="str">
+        <x:v>见竞争分析页与逐项来源</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3207,7 +3302,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d2458ac7b084278"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc82d75e25018428a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3675,7 +3770,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc66efe386964a34"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6176a40f3cbc4d78"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4184,7 +4279,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4576c6836ac64f29"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6a4041127c04795"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4306,16 +4401,16 @@
         <x:v>25%默认</x:v>
       </x:c>
       <x:c r="C8" s="21" t="str">
-        <x:v>1：评论／品牌／变体壁垒明显</x:v>
+        <x:v>1：集中、自营、评论或SKU壁垒明显</x:v>
       </x:c>
       <x:c r="D8" s="21" t="str">
-        <x:v>3：有新链接但进入点待验证</x:v>
+        <x:v>3：部分类目信号友好，词或店铺空间待验证</x:v>
       </x:c>
       <x:c r="E8" s="21" t="str">
-        <x:v>5：评论门槛低、新品活跃、有SKU缺口</x:v>
+        <x:v>5：类目机会、广告承受力、店铺／SKU空间有证据</x:v>
       </x:c>
       <x:c r="F8" s="21" t="str">
-        <x:v>初筛观察；深度判断看前20</x:v>
+        <x:v>初筛注明限制；深度看三层竞争及前20</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="76" customHeight="1">
@@ -4809,7 +4904,7 @@
         <x:v>2026-10-12T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="110" customHeight="1">
+    <x:row r="7" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A7" s="21" t="str">
         <x:v>软件选品法</x:v>
       </x:c>
@@ -4817,10 +4912,10 @@
         <x:v>发现渠道</x:v>
       </x:c>
       <x:c r="C7" s="21" t="str">
-        <x:v>Jungle Scout Product Database／Opportunity Finder 或卖家精灵；POE</x:v>
+        <x:v>Jungle Scout或卖家精灵；POE；Sorftime BSR（已有key）；无key用Flapen＋ASINSIGHT</x:v>
       </x:c>
       <x:c r="D7" s="21" t="str">
-        <x:v>按站点、价格、尺寸等筛选后核查商品页</x:v>
+        <x:v>按站点、价格、尺寸等筛选后核查商品页，分开记录类目BSR与关键词样本</x:v>
       </x:c>
       <x:c r="E7" s="21" t="str">
         <x:v>批量效率高、可比较多个维度</x:v>
@@ -4866,7 +4961,10 @@
       <x:c r="R7" s="21" t="str">
         <x:v>https://www.junglescout.com/features/product-database/
 https://www.sellersprite.com/cn
-https://sell.amazon.com/tools/product-opportunity-explorer</x:v>
+https://sell.amazon.com/tools/product-opportunity-explorer
+https://www.sorftime.com/en-US
+https://flapen.com/research/us
+https://www.asinsight.com/</x:v>
       </x:c>
       <x:c r="S7" s="24" t="d">
         <x:v>2026-10-12T00:00:00.000Z</x:v>
@@ -4934,7 +5032,7 @@
         <x:v>2026-10-12T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="110" customHeight="1">
+    <x:row r="9" ht="92.4000015258789" hidden="0" customHeight="1">
       <x:c r="A9" s="21" t="str">
         <x:v>关键词选品法</x:v>
       </x:c>
@@ -4942,7 +5040,7 @@
         <x:v>发现渠道</x:v>
       </x:c>
       <x:c r="C9" s="21" t="str">
-        <x:v>卖家精灵关键词选品／挖掘；Jungle Scout Keyword Scout；Google Trends／POE</x:v>
+        <x:v>卖家精灵／Jungle Scout Keyword Scout／ASINSIGHT；Google Trends／POE；Amazon广告后台建议竞价</x:v>
       </x:c>
       <x:c r="D9" s="21" t="str">
         <x:v>稳定、增长、长尾词分组，匹配买家意图</x:v>
@@ -4954,7 +5052,7 @@
         <x:v>搜索不等于购买，品牌词和小基数增长误导</x:v>
       </x:c>
       <x:c r="G9" s="21" t="str">
-        <x:v>核查绝对量、周期、相关性与商品结果</x:v>
+        <x:v>核查绝对量、周期、相关性；后台记录匹配类型、建议区间及币种，结合CVR复核利润承受力</x:v>
       </x:c>
       <x:c r="H9" s="21" t="str">
         <x:v>有类目或目标人群，研究细分需求</x:v>
@@ -4991,7 +5089,9 @@
       <x:c r="R9" s="21" t="str">
         <x:v>https://cn.sellersprite.com/cn/help/market-selection-guide
 https://support.junglescout.com/hc/en-us/articles/360008770253-Keyword-Scout
-https://support.google.com/trends/answer/4365533?hl=zh-Hans</x:v>
+https://support.google.com/trends/answer/4365533?hl=zh-Hans
+https://www.asinsight.com/
+https://advertising.amazon.com/library/guides/targeting-with-sponsored-products/</x:v>
       </x:c>
       <x:c r="S9" s="24" t="d">
         <x:v>2026-10-12T00:00:00.000Z</x:v>
@@ -5130,7 +5230,7 @@
         <x:v>发现渠道</x:v>
       </x:c>
       <x:c r="C12" s="21" t="str">
-        <x:v>Amazon卖家商品列表、品牌店铺、商品页；Keepa／卖家精灵辅助</x:v>
+        <x:v>Amazon卖家列表／品牌页；官方商标库；Keepa历史与网页推广查询</x:v>
       </x:c>
       <x:c r="D12" s="21" t="str">
         <x:v>比较能力相近店铺的新品、配件与产品组合</x:v>
@@ -5142,7 +5242,7 @@
         <x:v>成功样本偏差，看不到广告及实际利润</x:v>
       </x:c>
       <x:c r="G12" s="21" t="str">
-        <x:v>同时记录停滞款，首批就找具体差异</x:v>
+        <x:v>比较评价与星级、商标、公开地区、SKU、文案图片、站外链接；同时记录停滞款及切入点</x:v>
       </x:c>
       <x:c r="H12" s="21" t="str">
         <x:v>学习品类、找相邻产品</x:v>
@@ -5614,7 +5714,7 @@
         <x:v>2026-10-12T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="110" customHeight="1">
+    <x:row r="20" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A20" s="21" t="str">
         <x:v>竞品分析法</x:v>
       </x:c>
@@ -5622,19 +5722,19 @@
         <x:v>补充视角</x:v>
       </x:c>
       <x:c r="C20" s="21" t="str">
-        <x:v>Amazon前20、Jungle Scout／卖家精灵、POE；Excel</x:v>
+        <x:v>Sorftime BSR（已有key）；无key用Flapen＋ASINSIGHT；Amazon广告后台、店铺、Keepa与网页</x:v>
       </x:c>
       <x:c r="D20" s="21" t="str">
-        <x:v>核查评论壁垒、变体覆盖、新品与价格错配</x:v>
+        <x:v>类目Top100／Top50、核心词竞价、店铺实力三层分析；另做关键词前20壁垒、SKU、新品与错配</x:v>
       </x:c>
       <x:c r="E20" s="21" t="str">
         <x:v>直接支持进入空间判断</x:v>
       </x:c>
       <x:c r="F20" s="21" t="str">
-        <x:v>快照及父子体口径误导，公开信息不含利润</x:v>
+        <x:v>快照、父子体与垄断定义有差异；降级工具不一定覆盖所有指标，公开信息不含利润</x:v>
       </x:c>
       <x:c r="G20" s="21" t="str">
-        <x:v>统一口径并补差评、历史与自有方案成本</x:v>
+        <x:v>分别保存样本、阈值、seller ID去重与缺项；建议竞价不当实际CPC，历史变化不当站外推广证明</x:v>
       </x:c>
       <x:c r="H20" s="21" t="str">
         <x:v>贯穿全部方法的验证</x:v>
@@ -5670,7 +5770,12 @@
       <x:c r="R20" s="21" t="str">
         <x:v>https://sell.amazon.com/tools/product-opportunity-explorer
 https://www.junglescout.com/features/product-database/
-https://www.sellersprite.com/cn</x:v>
+https://www.sellersprite.com/cn
+https://www.sorftime.com/en-US
+https://flapen.com/research/us
+https://www.asinsight.com/
+https://advertising.amazon.com/library/guides/targeting-with-sponsored-products/
+https://keepa.com/</x:v>
       </x:c>
       <x:c r="S20" s="24" t="d">
         <x:v>2026-10-12T00:00:00.000Z</x:v>
@@ -5688,7 +5793,886 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R188b0ccf10084e7d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56c2398aa8a047f4"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF537682"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="27" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="31" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="42" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="52" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="42" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="32" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="48" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="17" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="14" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="58" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="2"/>
+      <x:c r="B1" s="2"/>
+      <x:c r="C1" s="2"/>
+      <x:c r="D1" s="2"/>
+      <x:c r="E1" s="2"/>
+      <x:c r="F1" s="2"/>
+      <x:c r="G1" s="2"/>
+      <x:c r="H1" s="2"/>
+      <x:c r="I1" s="2"/>
+      <x:c r="J1" s="2"/>
+      <x:c r="K1" s="2"/>
+      <x:c r="L1" s="2"/>
+      <x:c r="M1" s="2"/>
+      <x:c r="N1" s="2"/>
+      <x:c r="O1" s="2"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="3" t="str">
+        <x:v>类目、关键词与店铺竞争分析</x:v>
+      </x:c>
+      <x:c r="B2" s="2"/>
+      <x:c r="C2" s="2"/>
+      <x:c r="D2" s="2"/>
+      <x:c r="E2" s="2"/>
+      <x:c r="F2" s="2"/>
+      <x:c r="G2" s="2"/>
+      <x:c r="H2" s="2"/>
+      <x:c r="I2" s="2"/>
+      <x:c r="J2" s="2"/>
+      <x:c r="K2" s="2"/>
+      <x:c r="L2" s="2"/>
+      <x:c r="M2" s="2"/>
+      <x:c r="N2" s="2"/>
+      <x:c r="O2" s="2"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="2" t="str">
+        <x:v>用户规则。阈值只产生单项信号；完整覆盖与口径核验后再综合判断。</x:v>
+      </x:c>
+      <x:c r="B3" s="2"/>
+      <x:c r="C3" s="2"/>
+      <x:c r="D3" s="2"/>
+      <x:c r="E3" s="2"/>
+      <x:c r="F3" s="2"/>
+      <x:c r="G3" s="2"/>
+      <x:c r="H3" s="2"/>
+      <x:c r="I3" s="2"/>
+      <x:c r="J3" s="2"/>
+      <x:c r="K3" s="2"/>
+      <x:c r="L3" s="2"/>
+      <x:c r="M3" s="2"/>
+      <x:c r="N3" s="2"/>
+      <x:c r="O3" s="2"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="2" t="str">
+        <x:v>工具路径待记录；无Sorftime key时使用Flapen＋ASINSIGHT</x:v>
+      </x:c>
+      <x:c r="B4" s="2"/>
+      <x:c r="C4" s="2"/>
+      <x:c r="D4" s="2"/>
+      <x:c r="E4" s="2"/>
+      <x:c r="F4" s="2"/>
+      <x:c r="G4" s="2"/>
+      <x:c r="H4" s="2"/>
+      <x:c r="I4" s="2"/>
+      <x:c r="J4" s="2"/>
+      <x:c r="K4" s="2"/>
+      <x:c r="L4" s="2"/>
+      <x:c r="M4" s="2"/>
+      <x:c r="N4" s="2"/>
+      <x:c r="O4" s="2"/>
+    </x:row>
+    <x:row r="5" ht="42" customHeight="1">
+      <x:c r="A5" s="18" t="str">
+        <x:v>分析层级</x:v>
+      </x:c>
+      <x:c r="B5" s="19" t="str">
+        <x:v>选品分析方法</x:v>
+      </x:c>
+      <x:c r="C5" s="19" t="str">
+        <x:v>研究对象</x:v>
+      </x:c>
+      <x:c r="D5" s="19" t="str">
+        <x:v>指标</x:v>
+      </x:c>
+      <x:c r="E5" s="19" t="str">
+        <x:v>观察／数值</x:v>
+      </x:c>
+      <x:c r="F5" s="19" t="str">
+        <x:v>单位</x:v>
+      </x:c>
+      <x:c r="G5" s="19" t="str">
+        <x:v>样本范围</x:v>
+      </x:c>
+      <x:c r="H5" s="19" t="str">
+        <x:v>统计定义</x:v>
+      </x:c>
+      <x:c r="I5" s="19" t="str">
+        <x:v>数据覆盖</x:v>
+      </x:c>
+      <x:c r="J5" s="19" t="str">
+        <x:v>判断规则</x:v>
+      </x:c>
+      <x:c r="K5" s="19" t="str">
+        <x:v>信号／分析</x:v>
+      </x:c>
+      <x:c r="L5" s="19" t="str">
+        <x:v>数据来源</x:v>
+      </x:c>
+      <x:c r="M5" s="19" t="str">
+        <x:v>采集日期</x:v>
+      </x:c>
+      <x:c r="N5" s="19" t="str">
+        <x:v>数据状态</x:v>
+      </x:c>
+      <x:c r="O5" s="20" t="str">
+        <x:v>限制与缺口</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="60" customHeight="1">
+      <x:c r="A6" s="21" t="str">
+        <x:v>类目</x:v>
+      </x:c>
+      <x:c r="B6" s="21" t="str">
+        <x:v>方法一：BSR Top100</x:v>
+      </x:c>
+      <x:c r="C6" s="21"/>
+      <x:c r="D6" s="21" t="str">
+        <x:v>近3个月新品占比</x:v>
+      </x:c>
+      <x:c r="E6" s="27"/>
+      <x:c r="F6" s="22" t="str">
+        <x:v>比例</x:v>
+      </x:c>
+      <x:c r="G6" s="22"/>
+      <x:c r="H6" s="22"/>
+      <x:c r="I6" s="22" t="str">
+        <x:v>未知</x:v>
+      </x:c>
+      <x:c r="J6" s="21" t="str">
+        <x:v>≥10%：新手友好信号</x:v>
+      </x:c>
+      <x:c r="K6" s="21" t="str">
+        <x:f>IF(OR(OR(C6="",F6="",AND(NOT(ISNUMBER(E6)),E6=""),G6="",H6="",I6&lt;&gt;"完整",L6="",NOT(ISNUMBER(M6)),AND(N6&lt;&gt;"实测",N6&lt;&gt;"估算")),NOT(ISNUMBER(E6)),E6&lt;0,E6&gt;1),"待验证",IF(E6&gt;=0.1,"达到新手友好信号","未达到此项规则"))</x:f>
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="L6" s="22"/>
+      <x:c r="M6" s="23"/>
+      <x:c r="N6" s="22" t="str">
+        <x:v>待采集</x:v>
+      </x:c>
+      <x:c r="O6" s="22" t="str">
+        <x:v>待核验：完整Top100；日期覆盖100条；采集日前3个日历月，含边界</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="60" customHeight="1">
+      <x:c r="A7" s="21" t="str">
+        <x:v>类目</x:v>
+      </x:c>
+      <x:c r="B7" s="21" t="str">
+        <x:v>方法一：BSR Top100</x:v>
+      </x:c>
+      <x:c r="C7" s="21"/>
+      <x:c r="D7" s="21" t="str">
+        <x:v>近6个月新品占比</x:v>
+      </x:c>
+      <x:c r="E7" s="27"/>
+      <x:c r="F7" s="22" t="str">
+        <x:v>比例</x:v>
+      </x:c>
+      <x:c r="G7" s="22"/>
+      <x:c r="H7" s="22"/>
+      <x:c r="I7" s="22" t="str">
+        <x:v>未知</x:v>
+      </x:c>
+      <x:c r="J7" s="21" t="str">
+        <x:v>≥20%：新手友好信号</x:v>
+      </x:c>
+      <x:c r="K7" s="21" t="str">
+        <x:f>IF(OR(OR(C7="",F7="",AND(NOT(ISNUMBER(E7)),E7=""),G7="",H7="",I7&lt;&gt;"完整",L7="",NOT(ISNUMBER(M7)),AND(N7&lt;&gt;"实测",N7&lt;&gt;"估算")),NOT(ISNUMBER(E7)),E7&lt;0,E7&gt;1),"待验证",IF(E7&gt;=0.2,"达到新手友好信号","未达到此项规则"))</x:f>
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="L7" s="22"/>
+      <x:c r="M7" s="23"/>
+      <x:c r="N7" s="22" t="str">
+        <x:v>待采集</x:v>
+      </x:c>
+      <x:c r="O7" s="22" t="str">
+        <x:v>待核验：完整Top100；日期覆盖100条；采集日前6个日历月，含边界</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="60" customHeight="1">
+      <x:c r="A8" s="21" t="str">
+        <x:v>类目</x:v>
+      </x:c>
+      <x:c r="B8" s="21" t="str">
+        <x:v>方法一：BSR Top100</x:v>
+      </x:c>
+      <x:c r="C8" s="21"/>
+      <x:c r="D8" s="21" t="str">
+        <x:v>上架时间分布</x:v>
+      </x:c>
+      <x:c r="E8" s="22"/>
+      <x:c r="F8" s="22" t="str">
+        <x:v>观察</x:v>
+      </x:c>
+      <x:c r="G8" s="22"/>
+      <x:c r="H8" s="22"/>
+      <x:c r="I8" s="22" t="str">
+        <x:v>未知</x:v>
+      </x:c>
+      <x:c r="J8" s="21" t="str">
+        <x:v>新品占比越大，机会越多</x:v>
+      </x:c>
+      <x:c r="K8" s="21" t="str">
+        <x:f>IF(OR(C8="",F8="",AND(NOT(ISNUMBER(E8)),E8=""),G8="",H8="",I8&lt;&gt;"完整",L8="",NOT(ISNUMBER(M8)),AND(N8&lt;&gt;"实测",N8&lt;&gt;"估算")),"待验证","待分析方向性证据")</x:f>
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="L8" s="22"/>
+      <x:c r="M8" s="23"/>
+      <x:c r="N8" s="22" t="str">
+        <x:v>待采集</x:v>
+      </x:c>
+      <x:c r="O8" s="22" t="str">
+        <x:v>待核验：类目BSR Top100；3／6／12个月及更早；注明日期代理值</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="60" customHeight="1">
+      <x:c r="A9" s="21" t="str">
+        <x:v>类目</x:v>
+      </x:c>
+      <x:c r="B9" s="21" t="str">
+        <x:v>方法一：BSR Top100</x:v>
+      </x:c>
+      <x:c r="C9" s="21"/>
+      <x:c r="D9" s="21" t="str">
+        <x:v>评论时间分布</x:v>
+      </x:c>
+      <x:c r="E9" s="22"/>
+      <x:c r="F9" s="22" t="str">
+        <x:v>观察</x:v>
+      </x:c>
+      <x:c r="G9" s="22"/>
+      <x:c r="H9" s="22"/>
+      <x:c r="I9" s="22" t="str">
+        <x:v>未知</x:v>
+      </x:c>
+      <x:c r="J9" s="21" t="str">
+        <x:v>核实轴后解释左／右，轴未知则待验证</x:v>
+      </x:c>
+      <x:c r="K9" s="21" t="str">
+        <x:f>IF(OR(C9="",F9="",AND(NOT(ISNUMBER(E9)),E9=""),G9="",H9="",I9&lt;&gt;"完整",L9="",NOT(ISNUMBER(M9)),AND(N9&lt;&gt;"实测",N9&lt;&gt;"估算")),"待验证","待分析方向性证据")</x:f>
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="L9" s="22"/>
+      <x:c r="M9" s="23"/>
+      <x:c r="N9" s="22" t="str">
+        <x:v>待采集</x:v>
+      </x:c>
+      <x:c r="O9" s="22" t="str">
+        <x:v>待核验：类目BSR Top100；工具图表；注明横轴、时间方向、区间、统计对象</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="60" customHeight="1">
+      <x:c r="A10" s="21" t="str">
+        <x:v>类目</x:v>
+      </x:c>
+      <x:c r="B10" s="21" t="str">
+        <x:v>方法一：BSR Top100</x:v>
+      </x:c>
+      <x:c r="C10" s="21"/>
+      <x:c r="D10" s="21" t="str">
+        <x:v>评论数量分布</x:v>
+      </x:c>
+      <x:c r="E10" s="22"/>
+      <x:c r="F10" s="22" t="str">
+        <x:v>观察</x:v>
+      </x:c>
+      <x:c r="G10" s="22"/>
+      <x:c r="H10" s="22"/>
+      <x:c r="I10" s="22" t="str">
+        <x:v>未知</x:v>
+      </x:c>
+      <x:c r="J10" s="21" t="str">
+        <x:v>低评论区多竞争小，高评论区多竞争大</x:v>
+      </x:c>
+      <x:c r="K10" s="21" t="str">
+        <x:f>IF(OR(C10="",F10="",AND(NOT(ISNUMBER(E10)),E10=""),G10="",H10="",I10&lt;&gt;"完整",L10="",NOT(ISNUMBER(M10)),AND(N10&lt;&gt;"实测",N10&lt;&gt;"估算")),"待验证","待分析方向性证据")</x:f>
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="L10" s="22"/>
+      <x:c r="M10" s="23"/>
+      <x:c r="N10" s="22" t="str">
+        <x:v>待采集</x:v>
+      </x:c>
+      <x:c r="O10" s="22" t="str">
+        <x:v>待核验：类目BSR Top100；从低到高的分桶与各桶数量</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="60" customHeight="1">
+      <x:c r="A11" s="21" t="str">
+        <x:v>类目</x:v>
+      </x:c>
+      <x:c r="B11" s="21" t="str">
+        <x:v>方法一：BSR Top100</x:v>
+      </x:c>
+      <x:c r="C11" s="21"/>
+      <x:c r="D11" s="21" t="str">
+        <x:v>品牌垄断程度</x:v>
+      </x:c>
+      <x:c r="E11" s="27"/>
+      <x:c r="F11" s="22" t="str">
+        <x:v>比例</x:v>
+      </x:c>
+      <x:c r="G11" s="22"/>
+      <x:c r="H11" s="22"/>
+      <x:c r="I11" s="22" t="str">
+        <x:v>未知</x:v>
+      </x:c>
+      <x:c r="J11" s="21" t="str">
+        <x:v>&lt;45%：可接受</x:v>
+      </x:c>
+      <x:c r="K11" s="21" t="str">
+        <x:f>IF(OR(OR(C11="",F11="",AND(NOT(ISNUMBER(E11)),E11=""),G11="",H11="",I11&lt;&gt;"完整",L11="",NOT(ISNUMBER(M11)),AND(N11&lt;&gt;"实测",N11&lt;&gt;"估算")),NOT(ISNUMBER(E11)),E11&lt;0,E11&gt;1),"待验证",IF(E11&lt;0.45,"可接受","未达到此项规则"))</x:f>
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="L11" s="22"/>
+      <x:c r="M11" s="23"/>
+      <x:c r="N11" s="22" t="str">
+        <x:v>待采集</x:v>
+      </x:c>
+      <x:c r="O11" s="22" t="str">
+        <x:v>待核验：同站点同类目；工具原范围；填写品牌聚合范围、分子、分母及周期</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="60" customHeight="1">
+      <x:c r="A12" s="21" t="str">
+        <x:v>类目</x:v>
+      </x:c>
+      <x:c r="B12" s="21" t="str">
+        <x:v>方法一：BSR Top100</x:v>
+      </x:c>
+      <x:c r="C12" s="21"/>
+      <x:c r="D12" s="21" t="str">
+        <x:v>店铺垄断程度</x:v>
+      </x:c>
+      <x:c r="E12" s="27"/>
+      <x:c r="F12" s="22" t="str">
+        <x:v>比例</x:v>
+      </x:c>
+      <x:c r="G12" s="22"/>
+      <x:c r="H12" s="22"/>
+      <x:c r="I12" s="22" t="str">
+        <x:v>未知</x:v>
+      </x:c>
+      <x:c r="J12" s="21" t="str">
+        <x:v>&lt;45%：可接受</x:v>
+      </x:c>
+      <x:c r="K12" s="21" t="str">
+        <x:f>IF(OR(OR(C12="",F12="",AND(NOT(ISNUMBER(E12)),E12=""),G12="",H12="",I12&lt;&gt;"完整",L12="",NOT(ISNUMBER(M12)),AND(N12&lt;&gt;"实测",N12&lt;&gt;"估算")),NOT(ISNUMBER(E12)),E12&lt;0,E12&gt;1),"待验证",IF(E12&lt;0.45,"可接受","未达到此项规则"))</x:f>
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="L12" s="22"/>
+      <x:c r="M12" s="23"/>
+      <x:c r="N12" s="22" t="str">
+        <x:v>待采集</x:v>
+      </x:c>
+      <x:c r="O12" s="22" t="str">
+        <x:v>待核验：同站点同类目；工具原范围；填写seller ID聚合范围、分子、分母及周期</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="60" customHeight="1">
+      <x:c r="A13" s="21" t="str">
+        <x:v>类目</x:v>
+      </x:c>
+      <x:c r="B13" s="21" t="str">
+        <x:v>方法一：BSR Top100</x:v>
+      </x:c>
+      <x:c r="C13" s="21"/>
+      <x:c r="D13" s="21" t="str">
+        <x:v>Amazon自营占比</x:v>
+      </x:c>
+      <x:c r="E13" s="27"/>
+      <x:c r="F13" s="22" t="str">
+        <x:v>比例</x:v>
+      </x:c>
+      <x:c r="G13" s="22"/>
+      <x:c r="H13" s="22"/>
+      <x:c r="I13" s="22" t="str">
+        <x:v>未知</x:v>
+      </x:c>
+      <x:c r="J13" s="21" t="str">
+        <x:v>&lt;19%：有利信号</x:v>
+      </x:c>
+      <x:c r="K13" s="21" t="str">
+        <x:f>IF(OR(OR(C13="",F13="",AND(NOT(ISNUMBER(E13)),E13=""),G13="",H13="",I13&lt;&gt;"完整",L13="",NOT(ISNUMBER(M13)),AND(N13&lt;&gt;"实测",N13&lt;&gt;"估算")),NOT(ISNUMBER(E13)),E13&lt;0,E13&gt;1),"待验证",IF(E13&lt;0.19,"有利信号","未达到此项规则"))</x:f>
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="L13" s="22"/>
+      <x:c r="M13" s="23"/>
+      <x:c r="N13" s="22" t="str">
+        <x:v>待采集</x:v>
+      </x:c>
+      <x:c r="O13" s="22" t="str">
+        <x:v>待核验：类目BSR Top100；按实际销售方识别；FBA不等于自营</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="60" customHeight="1">
+      <x:c r="A14" s="21" t="str">
+        <x:v>类目</x:v>
+      </x:c>
+      <x:c r="B14" s="21" t="str">
+        <x:v>方法一：BSR Top100</x:v>
+      </x:c>
+      <x:c r="C14" s="21"/>
+      <x:c r="D14" s="21" t="str">
+        <x:v>FBM占比</x:v>
+      </x:c>
+      <x:c r="E14" s="27"/>
+      <x:c r="F14" s="22" t="str">
+        <x:v>比例</x:v>
+      </x:c>
+      <x:c r="G14" s="22"/>
+      <x:c r="H14" s="22"/>
+      <x:c r="I14" s="22" t="str">
+        <x:v>未知</x:v>
+      </x:c>
+      <x:c r="J14" s="21" t="str">
+        <x:v>越高越有利，无固定通过线</x:v>
+      </x:c>
+      <x:c r="K14" s="21" t="str">
+        <x:f>IF(OR(C14="",F14="",AND(NOT(ISNUMBER(E14)),E14=""),G14="",H14="",I14&lt;&gt;"完整",L14="",NOT(ISNUMBER(M14)),AND(N14&lt;&gt;"实测",N14&lt;&gt;"估算")),"待验证","待分析方向性证据")</x:f>
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="L14" s="22"/>
+      <x:c r="M14" s="23"/>
+      <x:c r="N14" s="22" t="str">
+        <x:v>待采集</x:v>
+      </x:c>
+      <x:c r="O14" s="22" t="str">
+        <x:v>待核验：类目BSR Top100；采集时代表卖家履约方式；注明比较基准</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="60" customHeight="1">
+      <x:c r="A15" s="21" t="str">
+        <x:v>类目</x:v>
+      </x:c>
+      <x:c r="B15" s="21" t="str">
+        <x:v>方法一：BSR Top100</x:v>
+      </x:c>
+      <x:c r="C15" s="21"/>
+      <x:c r="D15" s="21" t="str">
+        <x:v>A+视频占比</x:v>
+      </x:c>
+      <x:c r="E15" s="27"/>
+      <x:c r="F15" s="22" t="str">
+        <x:v>比例</x:v>
+      </x:c>
+      <x:c r="G15" s="22"/>
+      <x:c r="H15" s="22"/>
+      <x:c r="I15" s="22" t="str">
+        <x:v>未知</x:v>
+      </x:c>
+      <x:c r="J15" s="21" t="str">
+        <x:v>越少越有利，无固定通过线</x:v>
+      </x:c>
+      <x:c r="K15" s="21" t="str">
+        <x:f>IF(OR(C15="",F15="",AND(NOT(ISNUMBER(E15)),E15=""),G15="",H15="",I15&lt;&gt;"完整",L15="",NOT(ISNUMBER(M15)),AND(N15&lt;&gt;"实测",N15&lt;&gt;"估算")),"待验证","待分析方向性证据")</x:f>
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="L15" s="22"/>
+      <x:c r="M15" s="23"/>
+      <x:c r="N15" s="22" t="str">
+        <x:v>待采集</x:v>
+      </x:c>
+      <x:c r="O15" s="22" t="str">
+        <x:v>待核验：类目BSR Top100；注明原定义；A+、视频、两者同时分别记录</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="60" customHeight="1">
+      <x:c r="A16" s="21" t="str">
+        <x:v>类目</x:v>
+      </x:c>
+      <x:c r="B16" s="21" t="str">
+        <x:v>方法一：BSR Top100</x:v>
+      </x:c>
+      <x:c r="C16" s="21"/>
+      <x:c r="D16" s="21" t="str">
+        <x:v>整体商品星级</x:v>
+      </x:c>
+      <x:c r="E16" s="50"/>
+      <x:c r="F16" s="22" t="str">
+        <x:v>星</x:v>
+      </x:c>
+      <x:c r="G16" s="22"/>
+      <x:c r="H16" s="22"/>
+      <x:c r="I16" s="22" t="str">
+        <x:v>未知</x:v>
+      </x:c>
+      <x:c r="J16" s="21" t="str">
+        <x:v>越低越有改善机会，结合差评可解决性</x:v>
+      </x:c>
+      <x:c r="K16" s="21" t="str">
+        <x:f>IF(OR(C16="",F16="",AND(NOT(ISNUMBER(E16)),E16=""),G16="",H16="",I16&lt;&gt;"完整",L16="",NOT(ISNUMBER(M16)),AND(N16&lt;&gt;"实测",N16&lt;&gt;"估算")),"待验证","待分析方向性证据")</x:f>
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="L16" s="22"/>
+      <x:c r="M16" s="23"/>
+      <x:c r="N16" s="22" t="str">
+        <x:v>待采集</x:v>
+      </x:c>
+      <x:c r="O16" s="22" t="str">
+        <x:v>待核验：类目BSR Top100；简单平均或销量加权；注明有效数量</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="60" customHeight="1">
+      <x:c r="A17" s="21" t="str">
+        <x:v>类目</x:v>
+      </x:c>
+      <x:c r="B17" s="21" t="str">
+        <x:v>方法二：BSR Top50</x:v>
+      </x:c>
+      <x:c r="C17" s="21"/>
+      <x:c r="D17" s="21" t="str">
+        <x:v>评价数&lt;1000的去重卖家数</x:v>
+      </x:c>
+      <x:c r="E17" s="22"/>
+      <x:c r="F17" s="22" t="str">
+        <x:v>家</x:v>
+      </x:c>
+      <x:c r="G17" s="22"/>
+      <x:c r="H17" s="22"/>
+      <x:c r="I17" s="22" t="str">
+        <x:v>未知</x:v>
+      </x:c>
+      <x:c r="J17" s="21" t="str">
+        <x:v>&gt;20家：新手友好信号</x:v>
+      </x:c>
+      <x:c r="K17" s="21" t="str">
+        <x:f>IF(OR(OR(C17="",F17="",AND(NOT(ISNUMBER(E17)),E17=""),G17="",H17="",I17&lt;&gt;"完整",L17="",NOT(ISNUMBER(M17)),AND(N17&lt;&gt;"实测",N17&lt;&gt;"估算")),NOT(ISNUMBER(E17)),E17&lt;0,E17&gt;50),"待验证",IF(E17&gt;20,"达到新手友好信号","未达到此项规则"))</x:f>
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="L17" s="22"/>
+      <x:c r="M17" s="23"/>
+      <x:c r="N17" s="22" t="str">
+        <x:v>待采集</x:v>
+      </x:c>
+      <x:c r="O17" s="22" t="str">
+        <x:v>待核验：完整类目BSR Top50；seller ID去重；一个卖家最多计一次</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="60" customHeight="1">
+      <x:c r="A18" s="21" t="str">
+        <x:v>核心关键词</x:v>
+      </x:c>
+      <x:c r="B18" s="21" t="str">
+        <x:v>Amazon广告后台</x:v>
+      </x:c>
+      <x:c r="C18" s="21"/>
+      <x:c r="D18" s="21" t="str">
+        <x:v>关键词建议竞价／实际CPC</x:v>
+      </x:c>
+      <x:c r="E18" s="22"/>
+      <x:c r="F18" s="22"/>
+      <x:c r="G18" s="22"/>
+      <x:c r="H18" s="22"/>
+      <x:c r="I18" s="22" t="str">
+        <x:v>未知</x:v>
+      </x:c>
+      <x:c r="J18" s="21" t="str">
+        <x:v>比较竞价压力，再结合CVR核验利润</x:v>
+      </x:c>
+      <x:c r="K18" s="21" t="str">
+        <x:f>IF(OR(C18="",F18="",AND(NOT(ISNUMBER(E18)),E18=""),G18="",H18="",I18&lt;&gt;"完整",L18="",NOT(ISNUMBER(M18)),AND(N18&lt;&gt;"实测",N18&lt;&gt;"估算")),"待验证","待分析方向性证据")</x:f>
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="L18" s="22"/>
+      <x:c r="M18" s="23"/>
+      <x:c r="N18" s="22" t="str">
+        <x:v>待采集</x:v>
+      </x:c>
+      <x:c r="O18" s="22" t="str">
+        <x:v>待核验：同站点、同广告与匹配类型；词、建议区间或实际周期；币种和归因口径</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="60" customHeight="1">
+      <x:c r="A19" s="21" t="str">
+        <x:v>产品／店铺</x:v>
+      </x:c>
+      <x:c r="B19" s="21" t="str">
+        <x:v>商品页、卖家页</x:v>
+      </x:c>
+      <x:c r="C19" s="21"/>
+      <x:c r="D19" s="21" t="str">
+        <x:v>评论数量与星级</x:v>
+      </x:c>
+      <x:c r="E19" s="22"/>
+      <x:c r="F19" s="22" t="str">
+        <x:v>观察</x:v>
+      </x:c>
+      <x:c r="G19" s="22"/>
+      <x:c r="H19" s="22"/>
+      <x:c r="I19" s="22" t="str">
+        <x:v>未知</x:v>
+      </x:c>
+      <x:c r="J19" s="21" t="str">
+        <x:v>结合积累、增长、星级与重复差评</x:v>
+      </x:c>
+      <x:c r="K19" s="21" t="str">
+        <x:f>IF(OR(C19="",F19="",AND(NOT(ISNUMBER(E19)),E19=""),G19="",H19="",I19&lt;&gt;"完整",L19="",NOT(ISNUMBER(M19)),AND(N19&lt;&gt;"实测",N19&lt;&gt;"估算")),"待验证","待分析方向性证据")</x:f>
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="L19" s="22"/>
+      <x:c r="M19" s="23"/>
+      <x:c r="N19" s="22" t="str">
+        <x:v>待采集</x:v>
+      </x:c>
+      <x:c r="O19" s="22" t="str">
+        <x:v>待核验：代表竞品及同店产品；商品评价与店铺feedback分别记录</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="60" customHeight="1">
+      <x:c r="A20" s="21" t="str">
+        <x:v>产品／店铺</x:v>
+      </x:c>
+      <x:c r="B20" s="21" t="str">
+        <x:v>官方商标数据库、品牌页</x:v>
+      </x:c>
+      <x:c r="C20" s="21"/>
+      <x:c r="D20" s="21" t="str">
+        <x:v>品牌商标</x:v>
+      </x:c>
+      <x:c r="E20" s="22"/>
+      <x:c r="F20" s="22" t="str">
+        <x:v>观察</x:v>
+      </x:c>
+      <x:c r="G20" s="22"/>
+      <x:c r="H20" s="22"/>
+      <x:c r="I20" s="22" t="str">
+        <x:v>未知</x:v>
+      </x:c>
+      <x:c r="J20" s="21" t="str">
+        <x:v>判断品牌资源；A+不证明商标注册</x:v>
+      </x:c>
+      <x:c r="K20" s="21" t="str">
+        <x:f>IF(OR(C20="",F20="",AND(NOT(ISNUMBER(E20)),E20=""),G20="",H20="",I20&lt;&gt;"完整",L20="",NOT(ISNUMBER(M20)),AND(N20&lt;&gt;"实测",N20&lt;&gt;"估算")),"待验证","待分析方向性证据")</x:f>
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="L20" s="22"/>
+      <x:c r="M20" s="23"/>
+      <x:c r="N20" s="22" t="str">
+        <x:v>待采集</x:v>
+      </x:c>
+      <x:c r="O20" s="22" t="str">
+        <x:v>待核验：目标销售国家、品牌主体；权利人、状态、类目、查询来源</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="60" customHeight="1">
+      <x:c r="A21" s="21" t="str">
+        <x:v>产品／店铺</x:v>
+      </x:c>
+      <x:c r="B21" s="21" t="str">
+        <x:v>卖家公开公司信息</x:v>
+      </x:c>
+      <x:c r="C21" s="21"/>
+      <x:c r="D21" s="21" t="str">
+        <x:v>国家与地区</x:v>
+      </x:c>
+      <x:c r="E21" s="22"/>
+      <x:c r="F21" s="22" t="str">
+        <x:v>观察</x:v>
+      </x:c>
+      <x:c r="G21" s="22"/>
+      <x:c r="H21" s="22"/>
+      <x:c r="I21" s="22" t="str">
+        <x:v>未知</x:v>
+      </x:c>
+      <x:c r="J21" s="21" t="str">
+        <x:v>作为店铺证据，不单凭地区推断实力</x:v>
+      </x:c>
+      <x:c r="K21" s="21" t="str">
+        <x:f>IF(OR(C21="",F21="",AND(NOT(ISNUMBER(E21)),E21=""),G21="",H21="",I21&lt;&gt;"完整",L21="",NOT(ISNUMBER(M21)),AND(N21&lt;&gt;"实测",N21&lt;&gt;"估算")),"待验证","待分析方向性证据")</x:f>
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="L21" s="22"/>
+      <x:c r="M21" s="23"/>
+      <x:c r="N21" s="22" t="str">
+        <x:v>待采集</x:v>
+      </x:c>
+      <x:c r="O21" s="22" t="str">
+        <x:v>待核验：实际seller ID对应公司主体；公开主体、国家、地区与来源</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="60" customHeight="1">
+      <x:c r="A22" s="21" t="str">
+        <x:v>产品／店铺</x:v>
+      </x:c>
+      <x:c r="B22" s="21" t="str">
+        <x:v>卖家列表、品牌店铺</x:v>
+      </x:c>
+      <x:c r="C22" s="21"/>
+      <x:c r="D22" s="21" t="str">
+        <x:v>产品列表与SKU策略</x:v>
+      </x:c>
+      <x:c r="E22" s="22"/>
+      <x:c r="F22" s="22" t="str">
+        <x:v>观察</x:v>
+      </x:c>
+      <x:c r="G22" s="22"/>
+      <x:c r="H22" s="22"/>
+      <x:c r="I22" s="22" t="str">
+        <x:v>未知</x:v>
+      </x:c>
+      <x:c r="J22" s="21" t="str">
+        <x:v>识别覆盖强度与可切入空间</x:v>
+      </x:c>
+      <x:c r="K22" s="21" t="str">
+        <x:f>IF(OR(C22="",F22="",AND(NOT(ISNUMBER(E22)),E22=""),G22="",H22="",I22&lt;&gt;"完整",L22="",NOT(ISNUMBER(M22)),AND(N22&lt;&gt;"实测",N22&lt;&gt;"估算")),"待验证","待分析方向性证据")</x:f>
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="L22" s="22"/>
+      <x:c r="M22" s="23"/>
+      <x:c r="N22" s="22" t="str">
+        <x:v>待采集</x:v>
+      </x:c>
+      <x:c r="O22" s="22" t="str">
+        <x:v>待核验：所查店铺及在售列表；SKU数、类目集中、系列与新品；注明范围</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="60" customHeight="1">
+      <x:c r="A23" s="21" t="str">
+        <x:v>产品／店铺</x:v>
+      </x:c>
+      <x:c r="B23" s="21" t="str">
+        <x:v>商品详情页</x:v>
+      </x:c>
+      <x:c r="C23" s="21"/>
+      <x:c r="D23" s="21" t="str">
+        <x:v>文案、图片、A+与视频</x:v>
+      </x:c>
+      <x:c r="E23" s="22"/>
+      <x:c r="F23" s="22" t="str">
+        <x:v>观察</x:v>
+      </x:c>
+      <x:c r="G23" s="22"/>
+      <x:c r="H23" s="22"/>
+      <x:c r="I23" s="22" t="str">
+        <x:v>未知</x:v>
+      </x:c>
+      <x:c r="J23" s="21" t="str">
+        <x:v>指出可见差距与实现成本</x:v>
+      </x:c>
+      <x:c r="K23" s="21" t="str">
+        <x:f>IF(OR(C23="",F23="",AND(NOT(ISNUMBER(E23)),E23=""),G23="",H23="",I23&lt;&gt;"完整",L23="",NOT(ISNUMBER(M23)),AND(N23&lt;&gt;"实测",N23&lt;&gt;"估算")),"待验证","待分析方向性证据")</x:f>
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="L23" s="22"/>
+      <x:c r="M23" s="23"/>
+      <x:c r="N23" s="22" t="str">
+        <x:v>待采集</x:v>
+      </x:c>
+      <x:c r="O23" s="22" t="str">
+        <x:v>待核验：代表竞品及对应版本；本地化、卖点、适配、实拍、场景与内容</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="60" customHeight="1">
+      <x:c r="A24" s="21" t="str">
+        <x:v>产品／店铺</x:v>
+      </x:c>
+      <x:c r="B24" s="21" t="str">
+        <x:v>Keepa辅助、网页核查</x:v>
+      </x:c>
+      <x:c r="C24" s="21"/>
+      <x:c r="D24" s="21" t="str">
+        <x:v>站外推广</x:v>
+      </x:c>
+      <x:c r="E24" s="22"/>
+      <x:c r="F24" s="22" t="str">
+        <x:v>观察</x:v>
+      </x:c>
+      <x:c r="G24" s="22"/>
+      <x:c r="H24" s="22"/>
+      <x:c r="I24" s="22" t="str">
+        <x:v>未知</x:v>
+      </x:c>
+      <x:c r="J24" s="21" t="str">
+        <x:v>历史变化不证明站外；查不到不等于没有</x:v>
+      </x:c>
+      <x:c r="K24" s="21" t="str">
+        <x:f>IF(OR(C24="",F24="",AND(NOT(ISNUMBER(E24)),E24=""),G24="",H24="",I24&lt;&gt;"完整",L24="",NOT(ISNUMBER(M24)),AND(N24&lt;&gt;"实测",N24&lt;&gt;"估算")),"待验证","待分析方向性证据")</x:f>
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="L24" s="22"/>
+      <x:c r="M24" s="23"/>
+      <x:c r="N24" s="22" t="str">
+        <x:v>待采集</x:v>
+      </x:c>
+      <x:c r="O24" s="22" t="str">
+        <x:v>待核验：ASIN／品牌／产品名搜索；Keepa变化时间、搜索式、渠道、推广链接与类型</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="11">
+    <x:dataValidation type="decimal" operator="between" sqref="E6">
+      <x:formula1>0</x:formula1>
+      <x:formula2>1</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="decimal" operator="between" sqref="E7">
+      <x:formula1>0</x:formula1>
+      <x:formula2>1</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="decimal" operator="between" sqref="E11">
+      <x:formula1>0</x:formula1>
+      <x:formula2>1</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="decimal" operator="between" sqref="E12">
+      <x:formula1>0</x:formula1>
+      <x:formula2>1</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="decimal" operator="between" sqref="E13">
+      <x:formula1>0</x:formula1>
+      <x:formula2>1</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="decimal" operator="between" sqref="E14">
+      <x:formula1>0</x:formula1>
+      <x:formula2>1</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="decimal" operator="between" sqref="E15">
+      <x:formula1>0</x:formula1>
+      <x:formula2>1</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="decimal" operator="between" sqref="E16">
+      <x:formula1>0</x:formula1>
+      <x:formula2>5</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="between" sqref="E17">
+      <x:formula1>0</x:formula1>
+      <x:formula2>50</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="I6:I24">
+      <x:formula1>"完整,部分,未知"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="N6:N24">
+      <x:formula1>"实测,估算,假设,待采集"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2344781ce51549e6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>